<commit_message>
Wire up the new Proyecto dropdown and Otro Servicio column, split multi-line extras into rows, clarify amounts are sin IVA
- proyecto now resolves from the new dropdown (single_selectwyfgzjm)
  first, falling back to the old text/dropdown columns.
- otro_servicio_basico points at the new long_text column
  (long_textu2mzaeqt). Each line the Lider enters (Enter = new line)
  becomes its own row in Servicios Basicos, same as trabajos_previos,
  instead of one combined list item - the section already grows
  dynamically via ensure_simple_list_capacity, so it now scales with
  however many lines they type.
- PLANTILLA_ALCANCE_COTIZACION.xlsx: "Precio Unitario"/"Subtotal"
  headers and the instructions note now say amounts must be entered
  sin IVA.
</commit_message>
<xml_diff>
--- a/templates/PLANTILLA_ALCANCE_COTIZACION.xlsx
+++ b/templates/PLANTILLA_ALCANCE_COTIZACION.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-30828" yWindow="-4464" windowWidth="30936" windowHeight="16776" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cotizacion" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cotizacion" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -571,7 +571,7 @@
     <row r="2" ht="28.05" customHeight="1" s="15">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Llene una fila por cada renglón de su cotización. No modifique los encabezados ni el orden de las columnas. Cantidad y Precio Unitario deben ser números.</t>
+          <t>Llene una fila por cada renglon de su cotizacion. No modifique los encabezados ni el orden de las columnas. Cantidad y Precio Unitario deben ser numeros. Los montos deben ingresarse SIN IVA.</t>
         </is>
       </c>
     </row>
@@ -598,12 +598,12 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Precio Unitario</t>
+          <t>Precio Unitario (sin IVA)</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Subtotal</t>
+          <t>Subtotal (sin IVA)</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">

</xml_diff>